<commit_message>
Update quick reference with 8/26 document-review facts
Cutover Nov 13-16 target / Nov 20-23 backup; tenant bootstrap account
renamed WMPGCCHADMIN; decommission signer corrected to Kyle Manderfield;
AWS DNS managed by WMP; E911 test calls validated by WMP; device
conversion via RMM-pushed package or analyst USB with migration waves
eliminated; break-glass alerting decided as an Entra ID sign-in alert.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9SFx2c7BjowTfENYrpiQo
</commit_message>
<xml_diff>
--- a/deliverables/WMP/WMP__Design_Quick_Reference__20260825.xlsx
+++ b/deliverables/WMP/WMP__Design_Quick_Reference__20260825.xlsx
@@ -503,7 +503,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>All settled design facts and decisions at a glance. Sources: gap register Resolved Decisions (G-01–G-64) and the 8/25 discovery session. Full detail on the other sheets. 8/25/2026.</t>
+          <t>All settled design facts and decisions at a glance. Sources: gap register Resolved Decisions (G-01-G-64), the 8/25 discovery session, and the 8/26 document review. Updated 8/26/2026.</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Mid-November 2026, single cutover event (weekend); Essendis proposes candidate weekends (avoid Thanksgiving week)</t>
+          <t>November 13-16, 2026 (target); November 20-23 backup. Single cutover weekend (confirmed in doc review 8/26; matches the Asana schedule)</t>
         </is>
       </c>
     </row>
@@ -623,6 +623,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -723,7 +724,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>No standing Global Admins — all PIM-eligible; separate cadm- prefixed admin accounts; time-bound activation with MFA; Essendis access (Michael Schraepfer, Jeremy Cornwell) removed at handoff</t>
+          <t>No standing Global Admins — all PIM-eligible; separate cadm- prefixed admin accounts; tenant bootstrap account WMPGCCHADMIN@wisconsinmetalparts.com (renamed 8/26 to avoid collision with the WMPAdmin LAPS account); time-bound activation with MFA; Essendis access (Michael Schraepfer, Jeremy Cornwell) removed at handoff</t>
         </is>
       </c>
     </row>
@@ -739,6 +740,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -795,6 +797,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
@@ -883,10 +886,11 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Arctic Wolf (WMP's) needs GCC High visibility — WMP-owned; monitoring/alerting design out of engagement scope</t>
-        </is>
-      </c>
-    </row>
+          <t>Arctic Wolf (WMP's) needs GCC High visibility — WMP-owned; monitoring/alerting design out of engagement scope. Break-glass sign-in alerting decided (8/26): Microsoft Entra ID sign-in alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
@@ -1011,10 +1015,11 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>ForensIT profile mapping; in-office waves (all devices can come in); scripted via NinjaOne; app redeployment via NinjaOne</t>
-        </is>
-      </c>
-    </row>
+          <t>ForensIT profile mapping executed via an RMM-pushed package or by an analyst with a USB stick — no migration waves (eliminated per 8/26 review); devices can be brought in-office if required; app redeployment via NinjaOne</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
@@ -1071,6 +1076,7 @@
         </is>
       </c>
     </row>
+    <row r="58"/>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
@@ -1111,7 +1117,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Delivered and configured by CallTower; Essendis validates per-site test calls</t>
+          <t>Delivered and configured by CallTower; WMP validates per-site test calls as part of CallTower service validation (8/26 review)</t>
         </is>
       </c>
     </row>
@@ -1139,6 +1145,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
@@ -1203,7 +1210,7 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Hosted at AWS; TTL to 30 min from 5 days out; &lt;1 hr domain-release gap at cutover</t>
+          <t>Hosted at AWS, managed by WMP; TTL to 30 min from 5 days out; &lt;1 hr domain-release gap at cutover</t>
         </is>
       </c>
     </row>
@@ -1231,6 +1238,7 @@
         </is>
       </c>
     </row>
+    <row r="74"/>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
@@ -1271,7 +1279,7 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>7-day monitored hold; authorization signed by Kyle Mandersfield</t>
+          <t>7-day monitored hold; authorization signed by Kyle Manderfield</t>
         </is>
       </c>
     </row>
@@ -1287,6 +1295,7 @@
         </is>
       </c>
     </row>
+    <row r="80"/>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
@@ -2744,13 +2753,13 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>WMP (8/25, via chat): 7-day monitored hold; Kyle Mandersfield signs the decommission authorization.
+          <t>WMP (8/25, via chat): 7-day monitored hold; Kyle Manderfield signs the decommission authorization.
 Discovery (8/25): decommission sequencing is in flux - leaning post-cutover (as the design documents). Material reframing: on-prem Exchange 2016 is a MANAGEMENT platform only - all mailboxes and mail flow moved to M365 commercial previously - so decommission is hybrid-config/management-server removal, not a mail migration.</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Design update: the pre-removal monitored hold is 7 days and the decommission authorization is signed by Kyle Mandersfield (WMP). Essendis defines the residual-connection evidence check within that window.</t>
+          <t>Design update: the pre-removal monitored hold is 7 days and the decommission authorization is signed by Kyle Manderfield (WMP). Essendis defines the residual-connection evidence check within that window.</t>
         </is>
       </c>
     </row>

</xml_diff>